<commit_message>
Add learning-signals metrics, telemetry & Planeir docs
Introduce daily metrics, telemetry configuration and supporting migrations for the learning-signals service, plus new Planeir product docs. Adds Makefile `metrics` target to run the idempotent daily metrics runner. New files include telemetry event catalogs (v4/v5), thresholds.yaml, drizzle migrations and meta snapshots for module-versioning and metric snapshots, plus job runners (metrics-cli, metrics-runner, thresholds) and related package/app/server/schema updates. Several routes, privacy/erasure logic, telemetry ingestion, and tests were updated or added to wire metric snapshots, module versioning and tenant-aware signals. Also adds Planeir strategy and implementation docs (acquisition plan, implementation design & prompts) and an updated model workbook.
</commit_message>
<xml_diff>
--- a/Planeir_Model1_vs_Model2.xlsx
+++ b/Planeir_Model1_vs_Model2.xlsx
@@ -12,6 +12,8 @@
     <sheet name="Model 2 — Lead-Gen" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Model 1 — Adviser SaaS" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Side-by-Side" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Engine 1 — White-Label" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Blended Plan" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="130">
   <si>
     <t xml:space="preserve">Model 1 vs Model 2 — where the value lies</t>
   </si>
@@ -308,6 +310,111 @@
   </si>
   <si>
     <t xml:space="preserve">Venture outcomes: SmartAsset ~$1bn+ valuation; NerdWallet IPO; Credit Karma acquired by Intuit for $7.1bn — all consumer-finance funnels monetised via provider referrals.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Engine 1 — white-label API for advisers (early revenue)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Advisers embed your branded AI planning chat + Irish-tax visuals on their own site. It converts their traffic into qualified, pre-filled leads. Recurring B2B cash with no consumer CAC — live in months. Benchmarked to Planswell ($450+/mo, one adviser per lead, completed plan included).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Subscription per firm / month (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Planswell ~$450; adviser software £75–200. Mid = defensible</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One-off setup / onboarding fee (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optional; aids cashflow + commitment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leads generated per firm / year (value proof)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Justifies price: 40 leads worth £65+ each &gt;&gt; €3,600/yr sub</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Revenue by phase</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Year 1 (design partners)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Year 2 (Irish scale)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Year 3 (UK entry)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paying firms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MRR (subscriptions)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Annual recurring revenue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+ setup fees (new firms, indic.)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Why it's the easy first revenue: contracted, recurring, sold to an audience you already know (Brokers Ireland), no consumer CAC, and it seeds your future lead-buyers + training data.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blended plan — two engines, mix shifts to consumer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Engine 1 (white-label) is the reliable, no-CAC cash floor that funds the build. Engine 2 (consumer funnel) is CAC-contingent but is where scale and enterprise value come from. Rates pull from the 'Model 2 — Lead-Gen' sheet.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Year 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Year 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Year 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Engine 1: paying firms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Engine 1 revenue (white-label)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Engine 2: consumer visitors / yr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  consented leads</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  lead / referral revenue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  ad + affiliate revenue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Engine 2 revenue (consumer)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOTAL REVENUE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Engine 1 share (de-risked B2B)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What each phase must prove (for the next raise)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">White-label live with 10 design-partner firms + renewals; consumer content engine ranking on auto-enrolment terms; blended CAC &lt; lead value. Fund via Enterprise Ireland HPSU + angels.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Repeatable, cheap consumer acquisition (organic majority) + first employer/provider distribution deal; marketplace lead-quality proof (lead→appointment→client). Raise seed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UK entry for both engines; marketplace liquidity + net revenue retention on white-label; consumer scale to 1M+ visitors. Raise Series A on consumer growth + data moat.</t>
   </si>
 </sst>
 </file>
@@ -321,7 +428,7 @@
     <numFmt numFmtId="167" formatCode="\€#,##0.00"/>
     <numFmt numFmtId="168" formatCode="#,##0"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="20">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -436,6 +543,35 @@
       <family val="0"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF008000"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF008000"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="9"/>
+      <color rgb="FF1F3864"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="9">
     <fill>
@@ -536,7 +672,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="51">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -706,6 +842,38 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1720,4 +1888,434 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="B2:F17"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="22"/>
+  </cols>
+  <sheetData>
+    <row r="2" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B2" s="1" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B3" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B5" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B6" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="C6" s="11" t="n">
+        <v>300</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="F6" s="10"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B7" s="12" t="s">
+        <v>99</v>
+      </c>
+      <c r="C7" s="27" t="n">
+        <v>500</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>100</v>
+      </c>
+      <c r="F7" s="10"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B8" s="12" t="s">
+        <v>101</v>
+      </c>
+      <c r="C8" s="28" t="n">
+        <v>40</v>
+      </c>
+      <c r="E8" s="10" t="s">
+        <v>102</v>
+      </c>
+      <c r="F8" s="10"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B10" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
+    </row>
+    <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B11" s="43"/>
+      <c r="C11" s="15" t="s">
+        <v>104</v>
+      </c>
+      <c r="D11" s="15" t="s">
+        <v>105</v>
+      </c>
+      <c r="E11" s="15" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B12" s="16" t="s">
+        <v>107</v>
+      </c>
+      <c r="C12" s="17" t="n">
+        <v>10</v>
+      </c>
+      <c r="D12" s="17" t="n">
+        <v>60</v>
+      </c>
+      <c r="E12" s="17" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B13" s="16" t="s">
+        <v>108</v>
+      </c>
+      <c r="C13" s="21" t="n">
+        <f aca="false">C12*C6</f>
+        <v>3000</v>
+      </c>
+      <c r="D13" s="21" t="n">
+        <f aca="false">D12*C6</f>
+        <v>18000</v>
+      </c>
+      <c r="E13" s="21" t="n">
+        <f aca="false">E12*C6</f>
+        <v>60000</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B14" s="19" t="s">
+        <v>109</v>
+      </c>
+      <c r="C14" s="20" t="n">
+        <f aca="false">C12*C6*12</f>
+        <v>36000</v>
+      </c>
+      <c r="D14" s="20" t="n">
+        <f aca="false">D12*C6*12</f>
+        <v>216000</v>
+      </c>
+      <c r="E14" s="20" t="n">
+        <f aca="false">E12*C6*12</f>
+        <v>720000</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="16" t="s">
+        <v>110</v>
+      </c>
+      <c r="C15" s="21" t="n">
+        <f aca="false">C12*C7</f>
+        <v>5000</v>
+      </c>
+      <c r="D15" s="21" t="n">
+        <f aca="false">(D12-C12)*C7</f>
+        <v>25000</v>
+      </c>
+      <c r="E15" s="21" t="n">
+        <f aca="false">(E12-D12)*C7</f>
+        <v>70000</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B16" s="26" t="s">
+        <v>111</v>
+      </c>
+      <c r="C16" s="26"/>
+      <c r="D16" s="26"/>
+      <c r="E16" s="26"/>
+      <c r="F16" s="26"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="26"/>
+      <c r="C17" s="26"/>
+      <c r="D17" s="26"/>
+      <c r="E17" s="26"/>
+      <c r="F17" s="26"/>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="E8:F8"/>
+    <mergeCell ref="B16:F17"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="B2:F19"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="0" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="4"/>
+  </cols>
+  <sheetData>
+    <row r="2" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B2" s="1" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B3" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B5" s="43"/>
+      <c r="C5" s="44" t="s">
+        <v>114</v>
+      </c>
+      <c r="D5" s="44" t="s">
+        <v>115</v>
+      </c>
+      <c r="E5" s="44" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B6" s="45" t="s">
+        <v>117</v>
+      </c>
+      <c r="C6" s="17" t="n">
+        <v>10</v>
+      </c>
+      <c r="D6" s="17" t="n">
+        <v>60</v>
+      </c>
+      <c r="E6" s="17" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B7" s="22" t="s">
+        <v>118</v>
+      </c>
+      <c r="C7" s="23" t="n">
+        <f aca="false">C6*'Engine 1 — White-Label'!C6*12</f>
+        <v>36000</v>
+      </c>
+      <c r="D7" s="23" t="n">
+        <f aca="false">D6*'Engine 1 — White-Label'!C6*12</f>
+        <v>216000</v>
+      </c>
+      <c r="E7" s="23" t="n">
+        <f aca="false">E6*'Engine 1 — White-Label'!C6*12</f>
+        <v>720000</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B8" s="45" t="s">
+        <v>119</v>
+      </c>
+      <c r="C8" s="17" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D8" s="17" t="n">
+        <v>300000</v>
+      </c>
+      <c r="E8" s="17" t="n">
+        <v>1500000</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B9" s="16" t="s">
+        <v>120</v>
+      </c>
+      <c r="C9" s="18" t="n">
+        <f aca="false">C8*'Model 2 — Lead-Gen'!C6*'Model 2 — Lead-Gen'!C7</f>
+        <v>1500</v>
+      </c>
+      <c r="D9" s="18" t="n">
+        <f aca="false">D8*'Model 2 — Lead-Gen'!C6*'Model 2 — Lead-Gen'!C7</f>
+        <v>9000</v>
+      </c>
+      <c r="E9" s="18" t="n">
+        <f aca="false">E8*'Model 2 — Lead-Gen'!C6*'Model 2 — Lead-Gen'!C7</f>
+        <v>45000</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B10" s="46" t="s">
+        <v>121</v>
+      </c>
+      <c r="C10" s="47" t="n">
+        <f aca="false">C9*'Model 2 — Lead-Gen'!C8</f>
+        <v>120000</v>
+      </c>
+      <c r="D10" s="47" t="n">
+        <f aca="false">D9*'Model 2 — Lead-Gen'!C8</f>
+        <v>720000</v>
+      </c>
+      <c r="E10" s="47" t="n">
+        <f aca="false">E9*'Model 2 — Lead-Gen'!C8</f>
+        <v>3600000</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B11" s="46" t="s">
+        <v>122</v>
+      </c>
+      <c r="C11" s="47" t="n">
+        <f aca="false">C8*'Model 2 — Lead-Gen'!C9</f>
+        <v>25000</v>
+      </c>
+      <c r="D11" s="47" t="n">
+        <f aca="false">D8*'Model 2 — Lead-Gen'!C9</f>
+        <v>150000</v>
+      </c>
+      <c r="E11" s="47" t="n">
+        <f aca="false">E8*'Model 2 — Lead-Gen'!C9</f>
+        <v>750000</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B12" s="22" t="s">
+        <v>123</v>
+      </c>
+      <c r="C12" s="23" t="n">
+        <f aca="false">C10+C11</f>
+        <v>145000</v>
+      </c>
+      <c r="D12" s="23" t="n">
+        <f aca="false">D10+D11</f>
+        <v>870000</v>
+      </c>
+      <c r="E12" s="23" t="n">
+        <f aca="false">E10+E11</f>
+        <v>4350000</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B13" s="48" t="s">
+        <v>124</v>
+      </c>
+      <c r="C13" s="20" t="n">
+        <f aca="false">C7+C12</f>
+        <v>181000</v>
+      </c>
+      <c r="D13" s="20" t="n">
+        <f aca="false">D7+D12</f>
+        <v>1086000</v>
+      </c>
+      <c r="E13" s="20" t="n">
+        <f aca="false">E7+E12</f>
+        <v>5070000</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B14" s="16" t="s">
+        <v>125</v>
+      </c>
+      <c r="C14" s="24" t="n">
+        <f aca="false">C7/C13</f>
+        <v>0.198895027624309</v>
+      </c>
+      <c r="D14" s="24" t="n">
+        <f aca="false">D7/D13</f>
+        <v>0.198895027624309</v>
+      </c>
+      <c r="E14" s="24" t="n">
+        <f aca="false">E7/E13</f>
+        <v>0.142011834319527</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="C16" s="3"/>
+      <c r="D16" s="3"/>
+      <c r="E16" s="3"/>
+    </row>
+    <row r="17" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B17" s="49" t="s">
+        <v>114</v>
+      </c>
+      <c r="C17" s="50" t="s">
+        <v>127</v>
+      </c>
+      <c r="D17" s="50"/>
+      <c r="E17" s="50"/>
+    </row>
+    <row r="18" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B18" s="49" t="s">
+        <v>115</v>
+      </c>
+      <c r="C18" s="50" t="s">
+        <v>128</v>
+      </c>
+      <c r="D18" s="50"/>
+      <c r="E18" s="50"/>
+    </row>
+    <row r="19" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B19" s="49" t="s">
+        <v>116</v>
+      </c>
+      <c r="C19" s="50" t="s">
+        <v>129</v>
+      </c>
+      <c r="D19" s="50"/>
+      <c r="E19" s="50"/>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="C17:E17"/>
+    <mergeCell ref="C18:E18"/>
+    <mergeCell ref="C19:E19"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>